<commit_message>
new logs updates on the small questions
</commit_message>
<xml_diff>
--- a/DPRAMLP_solutions_comparison.xlsx
+++ b/DPRAMLP_solutions_comparison.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10402"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shouyuxie/MD_log/reImplement_Compress/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEFD51D8-FF0D-D247-9619-3FCB11294A0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB8659A1-634F-4849-A90A-39C4BE4C46B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51200" yWindow="17040" windowWidth="28800" windowHeight="16080" xr2:uid="{1505743E-F2C6-A645-9EC7-A56F67DC2BCC}"/>
+    <workbookView xWindow="4080" yWindow="720" windowWidth="46320" windowHeight="26680" activeTab="1" xr2:uid="{1505743E-F2C6-A645-9EC7-A56F67DC2BCC}"/>
   </bookViews>
   <sheets>
     <sheet name="Xfab DPRAM choices" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="17">
   <si>
     <t>Xfab dual port ram choices to buffer 2k lines of data</t>
   </si>
@@ -85,12 +86,15 @@
   <si>
     <t>Total one side height</t>
   </si>
+  <si>
+    <t>DPRAMLP size comparison</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -110,8 +114,15 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF006100"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -124,8 +135,13 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -133,11 +149,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -149,14 +181,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Good" xfId="1" builtinId="26"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1655,7 +1695,7 @@
   <dimension ref="A2:L28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="6" max="6" width="8.5" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" customWidth="1"/>
     <col min="7" max="7" width="13.33203125" customWidth="1"/>
     <col min="8" max="8" width="19.1640625" customWidth="1"/>
     <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
@@ -1663,14 +1703,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B3" s="1"/>
@@ -1752,14 +1792,14 @@
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -1959,7 +1999,7 @@
         <v>120.69965567999999</v>
       </c>
       <c r="L20">
-        <f t="shared" ref="L20:L25" si="3">D20*F20/2000</f>
+        <f t="shared" ref="L20" si="3">D20*F20/2000</f>
         <v>106.38080000000001</v>
       </c>
     </row>
@@ -1997,7 +2037,7 @@
         <v>121.19731711999999</v>
       </c>
       <c r="L21">
-        <f t="shared" ref="L21:L25" si="4">D21*F20/2000</f>
+        <f t="shared" ref="L21" si="4">D21*F20/2000</f>
         <v>60.339199999999998</v>
       </c>
     </row>
@@ -2055,7 +2095,7 @@
       <c r="E23" s="2">
         <v>0.84</v>
       </c>
-      <c r="F23" s="5">
+      <c r="F23" s="6">
         <v>128</v>
       </c>
       <c r="G23">
@@ -2095,7 +2135,7 @@
       <c r="E24" s="2">
         <v>0.89200000000000002</v>
       </c>
-      <c r="F24" s="5"/>
+      <c r="F24" s="6"/>
       <c r="G24">
         <f>E24*F23</f>
         <v>114.176</v>
@@ -2133,7 +2173,7 @@
       <c r="E25" s="2">
         <v>1.0740000000000001</v>
       </c>
-      <c r="F25" s="5"/>
+      <c r="F25" s="6"/>
       <c r="G25">
         <f>E25*F23</f>
         <v>137.47200000000001</v>
@@ -2175,7 +2215,7 @@
       <c r="E26" s="2">
         <v>1.6080000000000001</v>
       </c>
-      <c r="F26" s="5">
+      <c r="F26" s="6">
         <v>64</v>
       </c>
       <c r="G26">
@@ -2199,7 +2239,7 @@
         <v>106.83362304000001</v>
       </c>
       <c r="L26">
-        <f t="shared" ref="L26:L27" si="5">D26*F26/2000</f>
+        <f t="shared" ref="L26" si="5">D26*F26/2000</f>
         <v>28.316800000000001</v>
       </c>
     </row>
@@ -2215,7 +2255,7 @@
       <c r="E27" s="2">
         <v>1.7909999999999999</v>
       </c>
-      <c r="F27" s="5"/>
+      <c r="F27" s="6"/>
       <c r="G27">
         <f>E27*F26</f>
         <v>114.624</v>
@@ -2287,6 +2327,12 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="B23:B25"/>
+    <mergeCell ref="F23:F25"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="F26:F27"/>
     <mergeCell ref="A20:A22"/>
     <mergeCell ref="B20:B22"/>
     <mergeCell ref="F20:F22"/>
@@ -2295,14 +2341,90 @@
     <mergeCell ref="A17:A19"/>
     <mergeCell ref="B17:B19"/>
     <mergeCell ref="F17:F19"/>
-    <mergeCell ref="A23:A25"/>
-    <mergeCell ref="B23:B25"/>
-    <mergeCell ref="F23:F25"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="F26:F27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{264FE7EB-CE72-304D-9AFB-E4A69DB57628}">
+  <dimension ref="A2:E7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B2" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="9">
+        <v>2048</v>
+      </c>
+      <c r="B5" s="9">
+        <v>8</v>
+      </c>
+      <c r="C5" s="8">
+        <v>347.5</v>
+      </c>
+      <c r="D5" s="8">
+        <v>822.1</v>
+      </c>
+      <c r="E5" s="8">
+        <v>0.28499999999999998</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="9"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="8">
+        <v>564.70000000000005</v>
+      </c>
+      <c r="D6" s="8">
+        <v>462.5</v>
+      </c>
+      <c r="E6" s="8">
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="8">
+        <v>999.3</v>
+      </c>
+      <c r="D7" s="8">
+        <v>284.5</v>
+      </c>
+      <c r="E7" s="8">
+        <v>0.28100000000000003</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="B2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
updates on the experiments for the irregular bit width and length and the ram size
</commit_message>
<xml_diff>
--- a/DPRAMLP_solutions_comparison.xlsx
+++ b/DPRAMLP_solutions_comparison.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10402"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shouyuxie/MD_log/reImplement_Compress/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Back_up\MD_log\reImplementation_of_Compression_MD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB8659A1-634F-4849-A90A-39C4BE4C46B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1688A41D-B7C0-4104-BDAD-436304BA66CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4080" yWindow="720" windowWidth="46320" windowHeight="26680" activeTab="1" xr2:uid="{1505743E-F2C6-A645-9EC7-A56F67DC2BCC}"/>
+    <workbookView xWindow="41475" yWindow="1335" windowWidth="28800" windowHeight="15345" activeTab="1" xr2:uid="{1505743E-F2C6-A645-9EC7-A56F67DC2BCC}"/>
   </bookViews>
   <sheets>
     <sheet name="Xfab DPRAM choices" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
+    <sheet name="dimension varies by bit size" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -169,13 +169,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -187,11 +191,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1693,26 +1696,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6141C456-EA45-444E-8228-BB840FADC9C0}">
   <dimension ref="A2:L28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" customWidth="1"/>
-    <col min="8" max="8" width="19.1640625" customWidth="1"/>
+    <col min="6" max="6" width="10.8984375" customWidth="1"/>
+    <col min="7" max="7" width="13.3984375" customWidth="1"/>
+    <col min="8" max="8" width="19.09765625" customWidth="1"/>
     <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
     <col min="10" max="11" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="B2" s="5" t="s">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -1720,7 +1723,7 @@
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -1728,7 +1731,7 @@
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -1736,7 +1739,7 @@
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
@@ -1744,7 +1747,7 @@
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
     </row>
-    <row r="7" spans="1:12" ht="19" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" ht="18" x14ac:dyDescent="0.35">
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -1754,7 +1757,7 @@
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
@@ -1762,7 +1765,7 @@
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
@@ -1770,7 +1773,7 @@
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -1778,7 +1781,7 @@
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
@@ -1786,22 +1789,22 @@
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A14" s="5" t="s">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A14" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>2</v>
       </c>
@@ -1839,11 +1842,11 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A17" s="4">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A17" s="6">
         <v>2048</v>
       </c>
-      <c r="B17" s="4">
+      <c r="B17" s="6">
         <v>8</v>
       </c>
       <c r="C17">
@@ -1855,7 +1858,7 @@
       <c r="E17">
         <v>0.28499999999999998</v>
       </c>
-      <c r="F17" s="4">
+      <c r="F17" s="6">
         <v>512</v>
       </c>
       <c r="G17">
@@ -1883,9 +1886,9 @@
         <v>210.45760000000001</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A18" s="4"/>
-      <c r="B18" s="4"/>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A18" s="6"/>
+      <c r="B18" s="6"/>
       <c r="C18">
         <v>564.70000000000005</v>
       </c>
@@ -1895,7 +1898,7 @@
       <c r="E18">
         <v>0.26</v>
       </c>
-      <c r="F18" s="4"/>
+      <c r="F18" s="6"/>
       <c r="G18">
         <f>E18*F17</f>
         <v>133.12</v>
@@ -1921,9 +1924,9 @@
         <v>118.4</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A19" s="4"/>
-      <c r="B19" s="4"/>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A19" s="6"/>
+      <c r="B19" s="6"/>
       <c r="C19">
         <v>999.3</v>
       </c>
@@ -1933,7 +1936,7 @@
       <c r="E19">
         <v>0.28100000000000003</v>
       </c>
-      <c r="F19" s="4"/>
+      <c r="F19" s="6"/>
       <c r="G19">
         <f>E19*F17</f>
         <v>143.87200000000001</v>
@@ -1959,11 +1962,11 @@
         <v>72.831999999999994</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A20" s="4">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A20" s="6">
         <v>2048</v>
       </c>
-      <c r="B20" s="4">
+      <c r="B20" s="6">
         <v>16</v>
       </c>
       <c r="C20" s="2">
@@ -1975,7 +1978,7 @@
       <c r="E20">
         <v>0.46800000000000003</v>
       </c>
-      <c r="F20" s="4">
+      <c r="F20" s="6">
         <v>256</v>
       </c>
       <c r="G20">
@@ -2003,9 +2006,9 @@
         <v>106.38080000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A21" s="4"/>
-      <c r="B21" s="4"/>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A21" s="6"/>
+      <c r="B21" s="6"/>
       <c r="C21" s="2">
         <v>1004.3</v>
       </c>
@@ -2015,7 +2018,7 @@
       <c r="E21" s="2">
         <v>0.46700000000000003</v>
       </c>
-      <c r="F21" s="4"/>
+      <c r="F21" s="6"/>
       <c r="G21">
         <f>E21*F20</f>
         <v>119.55200000000001</v>
@@ -2041,9 +2044,9 @@
         <v>60.339199999999998</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4"/>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A22" s="6"/>
+      <c r="B22" s="6"/>
       <c r="C22" s="2">
         <v>1878.7</v>
       </c>
@@ -2053,7 +2056,7 @@
       <c r="E22" s="2">
         <v>0.53800000000000003</v>
       </c>
-      <c r="F22" s="4"/>
+      <c r="F22" s="6"/>
       <c r="G22">
         <f>E22*F20</f>
         <v>137.72800000000001</v>
@@ -2079,11 +2082,11 @@
         <v>37.567999999999998</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A23" s="4">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A23" s="6">
         <v>2048</v>
       </c>
-      <c r="B23" s="4">
+      <c r="B23" s="6">
         <v>32</v>
       </c>
       <c r="C23" s="2">
@@ -2095,7 +2098,7 @@
       <c r="E23" s="2">
         <v>0.84</v>
       </c>
-      <c r="F23" s="6">
+      <c r="F23" s="8">
         <v>128</v>
       </c>
       <c r="G23">
@@ -2123,9 +2126,9 @@
         <v>54.335999999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A24" s="4"/>
-      <c r="B24" s="4"/>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A24" s="6"/>
+      <c r="B24" s="6"/>
       <c r="C24" s="2">
         <v>1883.7</v>
       </c>
@@ -2135,7 +2138,7 @@
       <c r="E24" s="2">
         <v>0.89200000000000002</v>
       </c>
-      <c r="F24" s="6"/>
+      <c r="F24" s="8"/>
       <c r="G24">
         <f>E24*F23</f>
         <v>114.176</v>
@@ -2161,9 +2164,9 @@
         <v>31.3216</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A25" s="4"/>
-      <c r="B25" s="4"/>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A25" s="6"/>
+      <c r="B25" s="6"/>
       <c r="C25" s="2">
         <v>3637.4</v>
       </c>
@@ -2173,7 +2176,7 @@
       <c r="E25" s="2">
         <v>1.0740000000000001</v>
       </c>
-      <c r="F25" s="6"/>
+      <c r="F25" s="8"/>
       <c r="G25">
         <f>E25*F23</f>
         <v>137.47200000000001</v>
@@ -2199,11 +2202,11 @@
         <v>19.929599999999997</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A26" s="4">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A26" s="6">
         <v>2048</v>
       </c>
-      <c r="B26" s="4">
+      <c r="B26" s="6">
         <v>64</v>
       </c>
       <c r="C26" s="2">
@@ -2215,7 +2218,7 @@
       <c r="E26" s="2">
         <v>1.6080000000000001</v>
       </c>
-      <c r="F26" s="6">
+      <c r="F26" s="8">
         <v>64</v>
       </c>
       <c r="G26">
@@ -2243,9 +2246,9 @@
         <v>28.316800000000001</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A27" s="4"/>
-      <c r="B27" s="4"/>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A27" s="6"/>
+      <c r="B27" s="6"/>
       <c r="C27" s="2">
         <v>3642.4</v>
       </c>
@@ -2255,7 +2258,7 @@
       <c r="E27" s="2">
         <v>1.7909999999999999</v>
       </c>
-      <c r="F27" s="6"/>
+      <c r="F27" s="8"/>
       <c r="G27">
         <f>E27*F26</f>
         <v>114.624</v>
@@ -2281,7 +2284,7 @@
         <v>16.8064</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>2048</v>
       </c>
@@ -2349,82 +2352,269 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{264FE7EB-CE72-304D-9AFB-E4A69DB57628}">
-  <dimension ref="A2:E7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A2:E19"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B2" s="7" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B2" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="8" t="s">
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="9">
         <v>2048</v>
       </c>
       <c r="B5" s="9">
         <v>8</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="4">
         <v>347.5</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="4">
         <v>822.1</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="4">
         <v>0.28499999999999998</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="9"/>
       <c r="B6" s="9"/>
-      <c r="C6" s="8">
+      <c r="C6" s="4">
         <v>564.70000000000005</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="4">
         <v>462.5</v>
       </c>
-      <c r="E6" s="8">
+      <c r="E6" s="4">
         <v>0.26</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="9"/>
       <c r="B7" s="9"/>
-      <c r="C7" s="8">
+      <c r="C7" s="4">
         <v>999.3</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="4">
         <v>284.5</v>
       </c>
-      <c r="E7" s="8">
+      <c r="E7" s="4">
         <v>0.28100000000000003</v>
       </c>
     </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="9">
+        <v>2048</v>
+      </c>
+      <c r="B8" s="9">
+        <v>7</v>
+      </c>
+      <c r="C8" s="4">
+        <v>320</v>
+      </c>
+      <c r="D8" s="4">
+        <v>821</v>
+      </c>
+      <c r="E8" s="4">
+        <v>0.26200000000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="9"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="4">
+        <v>509.7</v>
+      </c>
+      <c r="D9" s="4">
+        <v>461.4</v>
+      </c>
+      <c r="E9" s="4">
+        <v>0.23400000000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="9"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="4">
+        <v>889.4</v>
+      </c>
+      <c r="D10" s="4">
+        <v>283.39999999999998</v>
+      </c>
+      <c r="E10" s="4">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="9">
+        <v>2048</v>
+      </c>
+      <c r="B11" s="9">
+        <v>6</v>
+      </c>
+      <c r="C11" s="4">
+        <v>292.5</v>
+      </c>
+      <c r="D11" s="4">
+        <v>819.9</v>
+      </c>
+      <c r="E11" s="4">
+        <v>0.23899999999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="9">
+        <v>2048</v>
+      </c>
+      <c r="B12" s="9"/>
+      <c r="C12" s="4">
+        <v>454.7</v>
+      </c>
+      <c r="D12" s="4">
+        <v>460.2</v>
+      </c>
+      <c r="E12" s="4">
+        <v>0.20899999999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="9"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="4">
+        <v>779.5</v>
+      </c>
+      <c r="D13" s="4">
+        <v>282.3</v>
+      </c>
+      <c r="E13" s="4">
+        <v>0.218</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="9">
+        <v>1024</v>
+      </c>
+      <c r="B14" s="9">
+        <v>16</v>
+      </c>
+      <c r="C14" s="4">
+        <v>564.70000000000005</v>
+      </c>
+      <c r="D14" s="4">
+        <v>481.7</v>
+      </c>
+      <c r="E14" s="4">
+        <v>0.26900000000000002</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="9"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="4">
+        <v>999.3</v>
+      </c>
+      <c r="D15" s="4">
+        <v>296.7</v>
+      </c>
+      <c r="E15" s="4">
+        <v>0.28999999999999998</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="9"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="4">
+        <v>1876</v>
+      </c>
+      <c r="D16" s="4">
+        <v>206.1</v>
+      </c>
+      <c r="E16" s="4">
+        <v>0.373</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="5">
+        <v>2032</v>
+      </c>
+      <c r="B17" s="5">
+        <v>8</v>
+      </c>
+      <c r="C17" s="4">
+        <v>347.5</v>
+      </c>
+      <c r="D17" s="4">
+        <v>816.7</v>
+      </c>
+      <c r="E17" s="4">
+        <v>0.28299999999999997</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="9">
+        <v>2016</v>
+      </c>
+      <c r="B18" s="9">
+        <v>8</v>
+      </c>
+      <c r="C18" s="4">
+        <v>347.5</v>
+      </c>
+      <c r="D18" s="4">
+        <v>811.2</v>
+      </c>
+      <c r="E18" s="4">
+        <v>0.28100000000000003</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="9"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="4">
+        <v>564.70000000000005</v>
+      </c>
+      <c r="D19" s="4">
+        <v>457</v>
+      </c>
+      <c r="E19" s="4">
+        <v>0.25700000000000001</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="11">
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="B14:B16"/>
     <mergeCell ref="A5:A7"/>
     <mergeCell ref="B5:B7"/>
-    <mergeCell ref="B2:D2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added FPGA choices we may ended up having
</commit_message>
<xml_diff>
--- a/DPRAMLP_solutions_comparison.xlsx
+++ b/DPRAMLP_solutions_comparison.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Back_up\MD_log\reImplementation_of_Compression_MD\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shouyuxie/MD_log/reImplement_Compress/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1688A41D-B7C0-4104-BDAD-436304BA66CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8F9AA8F-620B-C94E-8665-23ADCC68C778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41475" yWindow="1335" windowWidth="28800" windowHeight="15345" activeTab="1" xr2:uid="{1505743E-F2C6-A645-9EC7-A56F67DC2BCC}"/>
+    <workbookView xWindow="18120" yWindow="2120" windowWidth="36840" windowHeight="20900" activeTab="2" xr2:uid="{1505743E-F2C6-A645-9EC7-A56F67DC2BCC}"/>
   </bookViews>
   <sheets>
     <sheet name="Xfab DPRAM choices" sheetId="1" r:id="rId1"/>
     <sheet name="dimension varies by bit size" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="38">
   <si>
     <t>Xfab dual port ram choices to buffer 2k lines of data</t>
   </si>
@@ -88,13 +89,76 @@
   </si>
   <si>
     <t>DPRAMLP size comparison</t>
+  </si>
+  <si>
+    <t>FPGA choices for chip testing</t>
+  </si>
+  <si>
+    <t>FPGA model</t>
+  </si>
+  <si>
+    <t>FPGA chip</t>
+  </si>
+  <si>
+    <t>Chip family</t>
+  </si>
+  <si>
+    <t>General Pin #</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Digilent Genesys ZU-3EG</t>
+  </si>
+  <si>
+    <t>Zynq Ultrascale+ MPSoC</t>
+  </si>
+  <si>
+    <t>XCZU3EG-SFVC784-1-E</t>
+  </si>
+  <si>
+    <t>Digilent Nexys Video</t>
+  </si>
+  <si>
+    <t>$549</t>
+  </si>
+  <si>
+    <t>Artix-7</t>
+  </si>
+  <si>
+    <t>160-pin FMC LPC</t>
+  </si>
+  <si>
+    <t>XCZU7EV-1FBVB900E</t>
+  </si>
+  <si>
+    <t>Avnet UltraZed-EV SOM + Carrier Card</t>
+  </si>
+  <si>
+    <t>Zynq UltraScale+ EV</t>
+  </si>
+  <si>
+    <t>XC7A200T-1SBG484C</t>
+  </si>
+  <si>
+    <t>$1249</t>
+  </si>
+  <si>
+    <t>160-pin FMC LPC (less?)</t>
+  </si>
+  <si>
+    <t>152 user PL I/O pins</t>
+  </si>
+  <si>
+    <t>N/A</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -121,8 +185,28 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -140,8 +224,14 @@
         <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -164,12 +254,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -185,21 +286,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="2" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="4">
+    <cellStyle name="20% - Accent1" xfId="3" builtinId="30"/>
     <cellStyle name="Good" xfId="1" builtinId="26"/>
+    <cellStyle name="Linked Cell" xfId="2" builtinId="24"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1696,26 +1804,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6141C456-EA45-444E-8228-BB840FADC9C0}">
   <dimension ref="A2:L28"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="6" max="6" width="10.8984375" customWidth="1"/>
-    <col min="7" max="7" width="13.3984375" customWidth="1"/>
-    <col min="8" max="8" width="19.09765625" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" customWidth="1"/>
+    <col min="8" max="8" width="19.1640625" customWidth="1"/>
     <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
     <col min="10" max="11" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B2" s="7" t="s">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="B2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -1723,7 +1831,7 @@
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -1731,7 +1839,7 @@
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -1739,7 +1847,7 @@
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
@@ -1747,7 +1855,7 @@
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
     </row>
-    <row r="7" spans="1:12" ht="18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" ht="19" x14ac:dyDescent="0.25">
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -1757,7 +1865,7 @@
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
@@ -1765,7 +1873,7 @@
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
@@ -1773,7 +1881,7 @@
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -1781,7 +1889,7 @@
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
@@ -1789,22 +1897,22 @@
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A14" s="7" t="s">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A14" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>2</v>
       </c>
@@ -1842,7 +1950,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="6">
         <v>2048</v>
       </c>
@@ -1886,7 +1994,7 @@
         <v>210.45760000000001</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="6"/>
       <c r="B18" s="6"/>
       <c r="C18">
@@ -1924,7 +2032,7 @@
         <v>118.4</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="6"/>
       <c r="B19" s="6"/>
       <c r="C19">
@@ -1962,7 +2070,7 @@
         <v>72.831999999999994</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="6">
         <v>2048</v>
       </c>
@@ -2006,7 +2114,7 @@
         <v>106.38080000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="6"/>
       <c r="B21" s="6"/>
       <c r="C21" s="2">
@@ -2044,7 +2152,7 @@
         <v>60.339199999999998</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="6"/>
       <c r="B22" s="6"/>
       <c r="C22" s="2">
@@ -2082,7 +2190,7 @@
         <v>37.567999999999998</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="6">
         <v>2048</v>
       </c>
@@ -2098,7 +2206,7 @@
       <c r="E23" s="2">
         <v>0.84</v>
       </c>
-      <c r="F23" s="8">
+      <c r="F23" s="7">
         <v>128</v>
       </c>
       <c r="G23">
@@ -2126,7 +2234,7 @@
         <v>54.335999999999999</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="6"/>
       <c r="B24" s="6"/>
       <c r="C24" s="2">
@@ -2138,7 +2246,7 @@
       <c r="E24" s="2">
         <v>0.89200000000000002</v>
       </c>
-      <c r="F24" s="8"/>
+      <c r="F24" s="7"/>
       <c r="G24">
         <f>E24*F23</f>
         <v>114.176</v>
@@ -2164,7 +2272,7 @@
         <v>31.3216</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="6"/>
       <c r="B25" s="6"/>
       <c r="C25" s="2">
@@ -2176,7 +2284,7 @@
       <c r="E25" s="2">
         <v>1.0740000000000001</v>
       </c>
-      <c r="F25" s="8"/>
+      <c r="F25" s="7"/>
       <c r="G25">
         <f>E25*F23</f>
         <v>137.47200000000001</v>
@@ -2202,7 +2310,7 @@
         <v>19.929599999999997</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="6">
         <v>2048</v>
       </c>
@@ -2218,7 +2326,7 @@
       <c r="E26" s="2">
         <v>1.6080000000000001</v>
       </c>
-      <c r="F26" s="8">
+      <c r="F26" s="7">
         <v>64</v>
       </c>
       <c r="G26">
@@ -2246,7 +2354,7 @@
         <v>28.316800000000001</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="6"/>
       <c r="B27" s="6"/>
       <c r="C27" s="2">
@@ -2258,7 +2366,7 @@
       <c r="E27" s="2">
         <v>1.7909999999999999</v>
       </c>
-      <c r="F27" s="8"/>
+      <c r="F27" s="7"/>
       <c r="G27">
         <f>E27*F26</f>
         <v>114.624</v>
@@ -2284,7 +2392,7 @@
         <v>16.8064</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>2048</v>
       </c>
@@ -2330,12 +2438,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A23:A25"/>
-    <mergeCell ref="B23:B25"/>
-    <mergeCell ref="F23:F25"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="F26:F27"/>
     <mergeCell ref="A20:A22"/>
     <mergeCell ref="B20:B22"/>
     <mergeCell ref="F20:F22"/>
@@ -2344,6 +2446,12 @@
     <mergeCell ref="A17:A19"/>
     <mergeCell ref="B17:B19"/>
     <mergeCell ref="F17:F19"/>
+    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="B23:B25"/>
+    <mergeCell ref="F23:F25"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="F26:F27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2353,16 +2461,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{264FE7EB-CE72-304D-9AFB-E4A69DB57628}">
   <dimension ref="A2:E19"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B2" s="10" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B2" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
@@ -2379,11 +2487,11 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="9">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="10">
         <v>2048</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="10">
         <v>8</v>
       </c>
       <c r="C5" s="4">
@@ -2396,9 +2504,9 @@
         <v>0.28499999999999998</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="9"/>
-      <c r="B6" s="9"/>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="10"/>
+      <c r="B6" s="10"/>
       <c r="C6" s="4">
         <v>564.70000000000005</v>
       </c>
@@ -2409,9 +2517,9 @@
         <v>0.26</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="9"/>
-      <c r="B7" s="9"/>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="10"/>
+      <c r="B7" s="10"/>
       <c r="C7" s="4">
         <v>999.3</v>
       </c>
@@ -2422,11 +2530,11 @@
         <v>0.28100000000000003</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="9">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="10">
         <v>2048</v>
       </c>
-      <c r="B8" s="9">
+      <c r="B8" s="10">
         <v>7</v>
       </c>
       <c r="C8" s="4">
@@ -2439,9 +2547,9 @@
         <v>0.26200000000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="9"/>
-      <c r="B9" s="9"/>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="10"/>
+      <c r="B9" s="10"/>
       <c r="C9" s="4">
         <v>509.7</v>
       </c>
@@ -2452,9 +2560,9 @@
         <v>0.23400000000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="9"/>
-      <c r="B10" s="9"/>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="10"/>
+      <c r="B10" s="10"/>
       <c r="C10" s="4">
         <v>889.4</v>
       </c>
@@ -2465,11 +2573,11 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="9">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="10">
         <v>2048</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="10">
         <v>6</v>
       </c>
       <c r="C11" s="4">
@@ -2482,11 +2590,11 @@
         <v>0.23899999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="9">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" s="10">
         <v>2048</v>
       </c>
-      <c r="B12" s="9"/>
+      <c r="B12" s="10"/>
       <c r="C12" s="4">
         <v>454.7</v>
       </c>
@@ -2497,9 +2605,9 @@
         <v>0.20899999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="9"/>
-      <c r="B13" s="9"/>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="10"/>
+      <c r="B13" s="10"/>
       <c r="C13" s="4">
         <v>779.5</v>
       </c>
@@ -2510,11 +2618,11 @@
         <v>0.218</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="9">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="10">
         <v>1024</v>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="10">
         <v>16</v>
       </c>
       <c r="C14" s="4">
@@ -2527,9 +2635,9 @@
         <v>0.26900000000000002</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="9"/>
-      <c r="B15" s="9"/>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" s="10"/>
+      <c r="B15" s="10"/>
       <c r="C15" s="4">
         <v>999.3</v>
       </c>
@@ -2540,9 +2648,9 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="9"/>
-      <c r="B16" s="9"/>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" s="10"/>
+      <c r="B16" s="10"/>
       <c r="C16" s="4">
         <v>1876</v>
       </c>
@@ -2553,7 +2661,7 @@
         <v>0.373</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="5">
         <v>2032</v>
       </c>
@@ -2570,11 +2678,11 @@
         <v>0.28299999999999997</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="9">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="10">
         <v>2016</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="10">
         <v>8</v>
       </c>
       <c r="C18" s="4">
@@ -2587,9 +2695,9 @@
         <v>0.28100000000000003</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="9"/>
-      <c r="B19" s="9"/>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="10"/>
+      <c r="B19" s="10"/>
       <c r="C19" s="4">
         <v>564.70000000000005</v>
       </c>
@@ -2617,4 +2725,100 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{664C75E2-3377-0E4E-A688-ECF4587CB5B6}">
+  <dimension ref="A5:E11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="21.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+    </row>
+    <row r="6" spans="1:5" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B5:E5"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
added URL to each boards
</commit_message>
<xml_diff>
--- a/DPRAMLP_solutions_comparison.xlsx
+++ b/DPRAMLP_solutions_comparison.xlsx
@@ -1,19 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shouyuxie/MD_log/reImplement_Compress/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0F86487-4736-5D4A-B90E-B730251B09FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Xfab DPRAM choices" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="dimension varies by bit size" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="FPGA_choices" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Xfab DPRAM choices" sheetId="1" r:id="rId1"/>
+    <sheet name="dimension varies by bit size" sheetId="2" r:id="rId2"/>
+    <sheet name="FPGA_choices" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -22,162 +38,172 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="48">
-  <si>
-    <t xml:space="preserve">Xfab dual port ram choices to buffer 2k lines of data</t>
-  </si>
-  <si>
-    <t xml:space="preserve">...</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Assume each pixel has 2 bits of data:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Which is in total 8Mb/1MB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Words</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bits</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Width (um)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Heights (um)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Area (mm2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"># of blocks needed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Area in total (mm2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total one side width (mm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Heights (mm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One side area (mm2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Geometric area (mm2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total one side height</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DPRAMLP size comparison</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FPGA choices for chip testing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FPGA model</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FPGA chip</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chip family</t>
-  </si>
-  <si>
-    <t xml:space="preserve">General Pin #</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Price</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ref Images</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Digilent Genesys ZU-3EG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XCZU3EG-SFVC784-1-E</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zynq Ultrascale+ MPSoC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">160-pin FMC LPC (less?)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$1249</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Digilent Nexys Video</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XC7A200T-1SBG484C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Artix-7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$549</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Avnet UltraZed-EV SOM + Carrier Card</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XCZU7EV-1FBVB900E</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zynq UltraScale+ EV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">152 user PL I/O pins</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N/A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Opal Kelly XEM7310</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XC7A200T-1FBG484</t>
-  </si>
-  <si>
-    <t xml:space="preserve">124 I/O samtec</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Opal Kelly ECM1900</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XCZU7EG-1FFVC1156E</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="52">
+  <si>
+    <t>Xfab dual port ram choices to buffer 2k lines of data</t>
+  </si>
+  <si>
+    <t>...</t>
+  </si>
+  <si>
+    <t>Assume each pixel has 2 bits of data:</t>
+  </si>
+  <si>
+    <t>Which is in total 8Mb/1MB</t>
+  </si>
+  <si>
+    <t>Words</t>
+  </si>
+  <si>
+    <t>Bits</t>
+  </si>
+  <si>
+    <t>Width (um)</t>
+  </si>
+  <si>
+    <t>Heights (um)</t>
+  </si>
+  <si>
+    <t>Area (mm2)</t>
+  </si>
+  <si>
+    <t># of blocks needed</t>
+  </si>
+  <si>
+    <t>Area in total (mm2)</t>
+  </si>
+  <si>
+    <t>Total one side width (mm)</t>
+  </si>
+  <si>
+    <t>Heights (mm)</t>
+  </si>
+  <si>
+    <t>One side area (mm2)</t>
+  </si>
+  <si>
+    <t>Geometric area (mm2)</t>
+  </si>
+  <si>
+    <t>Total one side height</t>
+  </si>
+  <si>
+    <t>DPRAMLP size comparison</t>
+  </si>
+  <si>
+    <t>FPGA choices for chip testing</t>
+  </si>
+  <si>
+    <t>FPGA model</t>
+  </si>
+  <si>
+    <t>FPGA chip</t>
+  </si>
+  <si>
+    <t>Chip family</t>
+  </si>
+  <si>
+    <t>General Pin #</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Ref Images</t>
+  </si>
+  <si>
+    <t>Digilent Genesys ZU-3EG</t>
+  </si>
+  <si>
+    <t>XCZU3EG-SFVC784-1-E</t>
+  </si>
+  <si>
+    <t>Zynq Ultrascale+ MPSoC</t>
+  </si>
+  <si>
+    <t>160-pin FMC LPC (less?)</t>
+  </si>
+  <si>
+    <t>$1249</t>
+  </si>
+  <si>
+    <t>Digilent Nexys Video</t>
+  </si>
+  <si>
+    <t>XC7A200T-1SBG484C</t>
+  </si>
+  <si>
+    <t>Artix-7</t>
+  </si>
+  <si>
+    <t>$549</t>
+  </si>
+  <si>
+    <t>Avnet UltraZed-EV SOM + Carrier Card</t>
+  </si>
+  <si>
+    <t>XCZU7EV-1FBVB900E</t>
+  </si>
+  <si>
+    <t>Zynq UltraScale+ EV</t>
+  </si>
+  <si>
+    <t>152 user PL I/O pins</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Opal Kelly XEM7310</t>
+  </si>
+  <si>
+    <t>XC7A200T-1FBG484</t>
+  </si>
+  <si>
+    <t>124 I/O samtec</t>
+  </si>
+  <si>
+    <t>Opal Kelly ECM1900</t>
+  </si>
+  <si>
+    <t>XCZU7EG-1FFVC1156E</t>
   </si>
   <si>
     <t xml:space="preserve">248 I/O samtec </t>
   </si>
   <si>
-    <t xml:space="preserve">Opal Kelly XEM8305</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XCAU15P-2FFVB676E</t>
+    <t>Opal Kelly XEM8305</t>
+  </si>
+  <si>
+    <t>XCAU15P-2FFVB676E</t>
   </si>
   <si>
     <t xml:space="preserve">Artix UltraScale+ </t>
   </si>
   <si>
-    <t xml:space="preserve">123 I/O samtec</t>
+    <t>123 I/O samtec</t>
+  </si>
+  <si>
+    <t>https://opalkelly.com/wp-content/uploads/ECM1900-SlideDeck.pdf</t>
+  </si>
+  <si>
+    <t>https://opalkelly.com/wp-content/uploads/XEM7310-SlideDeck-1.pdf</t>
+  </si>
+  <si>
+    <t>https://opalkelly.com/wp-content/uploads/8305micropresentation-1.pdf</t>
+  </si>
+  <si>
+    <t>https://digilent.com/shop/genesys-zu-zynq-ultrascale-mpsoc-development-board/?srsltid=AfmBOoowYQII1o9UojQ6DLvITs0JYp-_c79JAWowi07v-pUHt2qhD9xG</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="General"/>
-    <numFmt numFmtId="166" formatCode="[$$-409]#,##0.00;[RED]\-[$$-409]#,##0.00"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]\-[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -186,25 +212,9 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
       <sz val="14"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
@@ -213,12 +223,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-      <family val="0"/>
     </font>
     <font>
       <sz val="12"/>
@@ -238,7 +242,21 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -257,26 +275,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.7999"/>
+        <fgColor theme="4" tint="0.79989013336588644"/>
         <bgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.5999"/>
+        <fgColor theme="9" tint="0.59987182226020086"/>
         <bgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
   </fills>
   <borders count="3">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
@@ -285,121 +303,74 @@
       </bottom>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="23">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+  <cellStyleXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+  </cellStyleXfs>
+  <cellXfs count="16">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-  </cellStyleXfs>
-  <cellXfs count="15">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="3" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="4"/>
   </cellXfs>
-  <cellStyles count="9">
+  <cellStyles count="5">
+    <cellStyle name="Excel Built-in 20% - Accent1" xfId="3" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
+    <cellStyle name="Excel Built-in Good" xfId="1" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+    <cellStyle name="Excel Built-in Linked Cell" xfId="2" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
+    <cellStyle name="Hyperlink" xfId="4" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="Excel Built-in Good" xfId="20"/>
-    <cellStyle name="Excel Built-in Linked Cell" xfId="21"/>
-    <cellStyle name="Excel Built-in 20% - Accent1" xfId="22"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -458,14 +429,30 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="twoCell">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>40320</xdr:colOff>
@@ -478,9 +465,15 @@
       <xdr:row>6</xdr:row>
       <xdr:rowOff>161280</xdr:rowOff>
     </xdr:to>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="0" name="Rectangle 2"/>
+        <xdr:cNvPr id="2" name="Rectangle 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -496,7 +489,7 @@
         </a:solidFill>
         <a:ln w="19050">
           <a:solidFill>
-            <a:srgbClr val="092a38"/>
+            <a:srgbClr val="092A38"/>
           </a:solidFill>
           <a:miter/>
         </a:ln>
@@ -518,7 +511,7 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>256320</xdr:colOff>
@@ -531,9 +524,15 @@
       <xdr:row>6</xdr:row>
       <xdr:rowOff>163800</xdr:rowOff>
     </xdr:to>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="1" name="Rectangle 3"/>
+        <xdr:cNvPr id="3" name="Rectangle 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -549,7 +548,7 @@
         </a:solidFill>
         <a:ln w="19050">
           <a:solidFill>
-            <a:srgbClr val="092a38"/>
+            <a:srgbClr val="092A38"/>
           </a:solidFill>
           <a:miter/>
         </a:ln>
@@ -571,7 +570,7 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>472320</xdr:colOff>
@@ -584,9 +583,15 @@
       <xdr:row>6</xdr:row>
       <xdr:rowOff>165960</xdr:rowOff>
     </xdr:to>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="Rectangle 4"/>
+        <xdr:cNvPr id="4" name="Rectangle 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -602,7 +607,7 @@
         </a:solidFill>
         <a:ln w="19050">
           <a:solidFill>
-            <a:srgbClr val="092a38"/>
+            <a:srgbClr val="092A38"/>
           </a:solidFill>
           <a:miter/>
         </a:ln>
@@ -624,7 +629,7 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>676440</xdr:colOff>
@@ -637,9 +642,15 @@
       <xdr:row>6</xdr:row>
       <xdr:rowOff>162360</xdr:rowOff>
     </xdr:to>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="Rectangle 5"/>
+        <xdr:cNvPr id="5" name="Rectangle 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000005000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -655,7 +666,7 @@
         </a:solidFill>
         <a:ln w="19050">
           <a:solidFill>
-            <a:srgbClr val="092a38"/>
+            <a:srgbClr val="092A38"/>
           </a:solidFill>
           <a:miter/>
         </a:ln>
@@ -677,7 +688,7 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>42840</xdr:colOff>
@@ -690,9 +701,15 @@
       <xdr:row>6</xdr:row>
       <xdr:rowOff>163800</xdr:rowOff>
     </xdr:to>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="4" name="Rectangle 6"/>
+        <xdr:cNvPr id="6" name="Rectangle 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000006000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -708,7 +725,7 @@
         </a:solidFill>
         <a:ln w="19050">
           <a:solidFill>
-            <a:srgbClr val="092a38"/>
+            <a:srgbClr val="092A38"/>
           </a:solidFill>
           <a:miter/>
         </a:ln>
@@ -730,7 +747,7 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>258480</xdr:colOff>
@@ -743,9 +760,15 @@
       <xdr:row>6</xdr:row>
       <xdr:rowOff>165960</xdr:rowOff>
     </xdr:to>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="5" name="Rectangle 7"/>
+        <xdr:cNvPr id="7" name="Rectangle 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000007000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -761,7 +784,7 @@
         </a:solidFill>
         <a:ln w="19050">
           <a:solidFill>
-            <a:srgbClr val="092a38"/>
+            <a:srgbClr val="092A38"/>
           </a:solidFill>
           <a:miter/>
         </a:ln>
@@ -783,7 +806,7 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>474480</xdr:colOff>
@@ -796,9 +819,15 @@
       <xdr:row>6</xdr:row>
       <xdr:rowOff>168120</xdr:rowOff>
     </xdr:to>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="6" name="Rectangle 8"/>
+        <xdr:cNvPr id="8" name="Rectangle 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000008000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -814,7 +843,7 @@
         </a:solidFill>
         <a:ln w="19050">
           <a:solidFill>
-            <a:srgbClr val="092a38"/>
+            <a:srgbClr val="092A38"/>
           </a:solidFill>
           <a:miter/>
         </a:ln>
@@ -836,7 +865,7 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>678960</xdr:colOff>
@@ -849,9 +878,15 @@
       <xdr:row>6</xdr:row>
       <xdr:rowOff>164880</xdr:rowOff>
     </xdr:to>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="7" name="Rectangle 9"/>
+        <xdr:cNvPr id="9" name="Rectangle 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000009000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -867,7 +902,7 @@
         </a:solidFill>
         <a:ln w="19050">
           <a:solidFill>
-            <a:srgbClr val="092a38"/>
+            <a:srgbClr val="092A38"/>
           </a:solidFill>
           <a:miter/>
         </a:ln>
@@ -889,7 +924,7 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>45000</xdr:colOff>
@@ -902,9 +937,15 @@
       <xdr:row>6</xdr:row>
       <xdr:rowOff>171720</xdr:rowOff>
     </xdr:to>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="8" name="Rectangle 10"/>
+        <xdr:cNvPr id="10" name="Rectangle 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000A000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -920,7 +961,7 @@
         </a:solidFill>
         <a:ln w="19050">
           <a:solidFill>
-            <a:srgbClr val="092a38"/>
+            <a:srgbClr val="092A38"/>
           </a:solidFill>
           <a:miter/>
         </a:ln>
@@ -942,7 +983,7 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>261000</xdr:colOff>
@@ -955,9 +996,15 @@
       <xdr:row>6</xdr:row>
       <xdr:rowOff>174240</xdr:rowOff>
     </xdr:to>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="9" name="Rectangle 11"/>
+        <xdr:cNvPr id="11" name="Rectangle 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000B000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -973,7 +1020,7 @@
         </a:solidFill>
         <a:ln w="19050">
           <a:solidFill>
-            <a:srgbClr val="092a38"/>
+            <a:srgbClr val="092A38"/>
           </a:solidFill>
           <a:miter/>
         </a:ln>
@@ -995,7 +1042,7 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>477000</xdr:colOff>
@@ -1008,9 +1055,15 @@
       <xdr:row>6</xdr:row>
       <xdr:rowOff>176400</xdr:rowOff>
     </xdr:to>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="10" name="Rectangle 12"/>
+        <xdr:cNvPr id="12" name="Rectangle 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000C000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -1026,7 +1079,7 @@
         </a:solidFill>
         <a:ln w="19050">
           <a:solidFill>
-            <a:srgbClr val="092a38"/>
+            <a:srgbClr val="092A38"/>
           </a:solidFill>
           <a:miter/>
         </a:ln>
@@ -1048,7 +1101,7 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>681120</xdr:colOff>
@@ -1061,9 +1114,15 @@
       <xdr:row>6</xdr:row>
       <xdr:rowOff>172800</xdr:rowOff>
     </xdr:to>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="11" name="Rectangle 13"/>
+        <xdr:cNvPr id="13" name="Rectangle 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000D000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -1079,7 +1138,7 @@
         </a:solidFill>
         <a:ln w="19050">
           <a:solidFill>
-            <a:srgbClr val="092a38"/>
+            <a:srgbClr val="092A38"/>
           </a:solidFill>
           <a:miter/>
         </a:ln>
@@ -1101,7 +1160,7 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>249120</xdr:colOff>
@@ -1114,9 +1173,15 @@
       <xdr:row>11</xdr:row>
       <xdr:rowOff>9360</xdr:rowOff>
     </xdr:to>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="12" name="Rounded Rectangle 14"/>
+        <xdr:cNvPr id="14" name="Rounded Rectangle 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000E000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -1130,11 +1195,11 @@
           </a:avLst>
         </a:prstGeom>
         <a:solidFill>
-          <a:srgbClr val="f6c6ad"/>
+          <a:srgbClr val="F6C6AD"/>
         </a:solidFill>
         <a:ln w="19050">
           <a:solidFill>
-            <a:srgbClr val="092a38"/>
+            <a:srgbClr val="092A38"/>
           </a:solidFill>
           <a:miter/>
         </a:ln>
@@ -1154,9 +1219,10 @@
         <a:fontRef idx="minor"/>
       </xdr:style>
       <xdr:txBody>
-        <a:bodyPr horzOverflow="clip" vertOverflow="clip" lIns="90000" rIns="90000" tIns="45000" bIns="45000" anchor="t">
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="90000" tIns="45000" rIns="90000" bIns="45000" anchor="t">
           <a:noAutofit/>
         </a:bodyPr>
+        <a:lstStyle/>
         <a:p>
           <a:pPr>
             <a:lnSpc>
@@ -1164,7 +1230,7 @@
             </a:lnSpc>
           </a:pPr>
           <a:r>
-            <a:rPr b="0" lang="en-GB" sz="1100" spc="-1" strike="noStrike">
+            <a:rPr lang="en-GB" sz="1100" b="0" strike="noStrike" spc="-1">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
@@ -1172,7 +1238,7 @@
             </a:rPr>
             <a:t>RAM</a:t>
           </a:r>
-          <a:endParaRPr b="0" lang="en-US" sz="1100" spc="-1" strike="noStrike">
+          <a:endParaRPr lang="en-US" sz="1100" b="0" strike="noStrike" spc="-1">
             <a:latin typeface="Times New Roman"/>
           </a:endParaRPr>
         </a:p>
@@ -1180,7 +1246,7 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>280440</xdr:colOff>
@@ -1193,9 +1259,15 @@
       <xdr:row>11</xdr:row>
       <xdr:rowOff>6120</xdr:rowOff>
     </xdr:to>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="13" name="Rounded Rectangle 15"/>
+        <xdr:cNvPr id="15" name="Rounded Rectangle 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000F000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -1209,11 +1281,11 @@
           </a:avLst>
         </a:prstGeom>
         <a:solidFill>
-          <a:srgbClr val="f6c6ad"/>
+          <a:srgbClr val="F6C6AD"/>
         </a:solidFill>
         <a:ln w="19050">
           <a:solidFill>
-            <a:srgbClr val="092a38"/>
+            <a:srgbClr val="092A38"/>
           </a:solidFill>
           <a:miter/>
         </a:ln>
@@ -1233,9 +1305,10 @@
         <a:fontRef idx="minor"/>
       </xdr:style>
       <xdr:txBody>
-        <a:bodyPr horzOverflow="clip" vertOverflow="clip" lIns="90000" rIns="90000" tIns="45000" bIns="45000" anchor="t">
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="90000" tIns="45000" rIns="90000" bIns="45000" anchor="t">
           <a:noAutofit/>
         </a:bodyPr>
+        <a:lstStyle/>
         <a:p>
           <a:pPr>
             <a:lnSpc>
@@ -1243,7 +1316,7 @@
             </a:lnSpc>
           </a:pPr>
           <a:r>
-            <a:rPr b="0" lang="en-GB" sz="1100" spc="-1" strike="noStrike">
+            <a:rPr lang="en-GB" sz="1100" b="0" strike="noStrike" spc="-1">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
@@ -1251,7 +1324,7 @@
             </a:rPr>
             <a:t>RAM</a:t>
           </a:r>
-          <a:endParaRPr b="0" lang="en-US" sz="1100" spc="-1" strike="noStrike">
+          <a:endParaRPr lang="en-US" sz="1100" b="0" strike="noStrike" spc="-1">
             <a:latin typeface="Times New Roman"/>
           </a:endParaRPr>
         </a:p>
@@ -1259,7 +1332,7 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>27720</xdr:colOff>
@@ -1272,9 +1345,15 @@
       <xdr:row>9</xdr:row>
       <xdr:rowOff>172080</xdr:rowOff>
     </xdr:to>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="14" name="Rounded Rectangle 16"/>
+        <xdr:cNvPr id="16" name="Rounded Rectangle 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000010000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -1288,11 +1367,11 @@
           </a:avLst>
         </a:prstGeom>
         <a:solidFill>
-          <a:srgbClr val="f6c6ad"/>
+          <a:srgbClr val="F6C6AD"/>
         </a:solidFill>
         <a:ln w="19050">
           <a:solidFill>
-            <a:srgbClr val="092a38"/>
+            <a:srgbClr val="092A38"/>
           </a:solidFill>
           <a:miter/>
         </a:ln>
@@ -1312,9 +1391,10 @@
         <a:fontRef idx="minor"/>
       </xdr:style>
       <xdr:txBody>
-        <a:bodyPr horzOverflow="clip" vertOverflow="clip" lIns="90000" rIns="90000" tIns="45000" bIns="45000" anchor="t">
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="90000" tIns="45000" rIns="90000" bIns="45000" anchor="t">
           <a:noAutofit/>
         </a:bodyPr>
+        <a:lstStyle/>
         <a:p>
           <a:pPr>
             <a:lnSpc>
@@ -1322,7 +1402,7 @@
             </a:lnSpc>
           </a:pPr>
           <a:r>
-            <a:rPr b="0" lang="en-GB" sz="1100" spc="-1" strike="noStrike">
+            <a:rPr lang="en-GB" sz="1100" b="0" strike="noStrike" spc="-1">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
@@ -1330,7 +1410,7 @@
             </a:rPr>
             <a:t>RAM</a:t>
           </a:r>
-          <a:endParaRPr b="0" lang="en-US" sz="1100" spc="-1" strike="noStrike">
+          <a:endParaRPr lang="en-US" sz="1100" b="0" strike="noStrike" spc="-1">
             <a:latin typeface="Times New Roman"/>
           </a:endParaRPr>
         </a:p>
@@ -1338,7 +1418,7 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>41400</xdr:colOff>
@@ -1351,9 +1431,15 @@
       <xdr:row>4</xdr:row>
       <xdr:rowOff>139320</xdr:rowOff>
     </xdr:to>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="15" name="Rounded Rectangle 17"/>
+        <xdr:cNvPr id="17" name="Rounded Rectangle 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000011000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -1367,11 +1453,11 @@
           </a:avLst>
         </a:prstGeom>
         <a:solidFill>
-          <a:srgbClr val="f6c6ad"/>
+          <a:srgbClr val="F6C6AD"/>
         </a:solidFill>
         <a:ln w="19050">
           <a:solidFill>
-            <a:srgbClr val="092a38"/>
+            <a:srgbClr val="092A38"/>
           </a:solidFill>
           <a:miter/>
         </a:ln>
@@ -1391,9 +1477,10 @@
         <a:fontRef idx="minor"/>
       </xdr:style>
       <xdr:txBody>
-        <a:bodyPr horzOverflow="clip" vertOverflow="clip" lIns="90000" rIns="90000" tIns="45000" bIns="45000" anchor="t">
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="90000" tIns="45000" rIns="90000" bIns="45000" anchor="t">
           <a:noAutofit/>
         </a:bodyPr>
+        <a:lstStyle/>
         <a:p>
           <a:pPr>
             <a:lnSpc>
@@ -1401,7 +1488,7 @@
             </a:lnSpc>
           </a:pPr>
           <a:r>
-            <a:rPr b="0" lang="en-GB" sz="1100" spc="-1" strike="noStrike">
+            <a:rPr lang="en-GB" sz="1100" b="0" strike="noStrike" spc="-1">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
@@ -1409,7 +1496,7 @@
             </a:rPr>
             <a:t>RAM</a:t>
           </a:r>
-          <a:endParaRPr b="0" lang="en-US" sz="1100" spc="-1" strike="noStrike">
+          <a:endParaRPr lang="en-US" sz="1100" b="0" strike="noStrike" spc="-1">
             <a:latin typeface="Times New Roman"/>
           </a:endParaRPr>
         </a:p>
@@ -1417,7 +1504,7 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>20880</xdr:colOff>
@@ -1430,9 +1517,15 @@
       <xdr:row>4</xdr:row>
       <xdr:rowOff>136080</xdr:rowOff>
     </xdr:to>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="16" name="Rounded Rectangle 18"/>
+        <xdr:cNvPr id="18" name="Rounded Rectangle 18">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000012000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -1446,11 +1539,11 @@
           </a:avLst>
         </a:prstGeom>
         <a:solidFill>
-          <a:srgbClr val="f6c6ad"/>
+          <a:srgbClr val="F6C6AD"/>
         </a:solidFill>
         <a:ln w="19050">
           <a:solidFill>
-            <a:srgbClr val="092a38"/>
+            <a:srgbClr val="092A38"/>
           </a:solidFill>
           <a:miter/>
         </a:ln>
@@ -1470,9 +1563,10 @@
         <a:fontRef idx="minor"/>
       </xdr:style>
       <xdr:txBody>
-        <a:bodyPr horzOverflow="clip" vertOverflow="clip" lIns="90000" rIns="90000" tIns="45000" bIns="45000" anchor="t">
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="90000" tIns="45000" rIns="90000" bIns="45000" anchor="t">
           <a:noAutofit/>
         </a:bodyPr>
+        <a:lstStyle/>
         <a:p>
           <a:pPr>
             <a:lnSpc>
@@ -1480,7 +1574,7 @@
             </a:lnSpc>
           </a:pPr>
           <a:r>
-            <a:rPr b="0" lang="en-GB" sz="1100" spc="-1" strike="noStrike">
+            <a:rPr lang="en-GB" sz="1100" b="0" strike="noStrike" spc="-1">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
@@ -1488,7 +1582,7 @@
             </a:rPr>
             <a:t>RAM</a:t>
           </a:r>
-          <a:endParaRPr b="0" lang="en-US" sz="1100" spc="-1" strike="noStrike">
+          <a:endParaRPr lang="en-US" sz="1100" b="0" strike="noStrike" spc="-1">
             <a:latin typeface="Times New Roman"/>
           </a:endParaRPr>
         </a:p>
@@ -1496,7 +1590,7 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>28800</xdr:colOff>
@@ -1509,9 +1603,15 @@
       <xdr:row>4</xdr:row>
       <xdr:rowOff>126720</xdr:rowOff>
     </xdr:to>
-    <xdr:sp>
+    <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="17" name="Rounded Rectangle 19"/>
+        <xdr:cNvPr id="19" name="Rounded Rectangle 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000013000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -1525,11 +1625,11 @@
           </a:avLst>
         </a:prstGeom>
         <a:solidFill>
-          <a:srgbClr val="f6c6ad"/>
+          <a:srgbClr val="F6C6AD"/>
         </a:solidFill>
         <a:ln w="19050">
           <a:solidFill>
-            <a:srgbClr val="092a38"/>
+            <a:srgbClr val="092A38"/>
           </a:solidFill>
           <a:miter/>
         </a:ln>
@@ -1549,9 +1649,10 @@
         <a:fontRef idx="minor"/>
       </xdr:style>
       <xdr:txBody>
-        <a:bodyPr horzOverflow="clip" vertOverflow="clip" lIns="90000" rIns="90000" tIns="45000" bIns="45000" anchor="t">
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="90000" tIns="45000" rIns="90000" bIns="45000" anchor="t">
           <a:noAutofit/>
         </a:bodyPr>
+        <a:lstStyle/>
         <a:p>
           <a:pPr>
             <a:lnSpc>
@@ -1559,7 +1660,7 @@
             </a:lnSpc>
           </a:pPr>
           <a:r>
-            <a:rPr b="0" lang="en-GB" sz="1100" spc="-1" strike="noStrike">
+            <a:rPr lang="en-GB" sz="1100" b="0" strike="noStrike" spc="-1">
               <a:solidFill>
                 <a:srgbClr val="000000"/>
               </a:solidFill>
@@ -1567,7 +1668,7 @@
             </a:rPr>
             <a:t>RAM</a:t>
           </a:r>
-          <a:endParaRPr b="0" lang="en-US" sz="1100" spc="-1" strike="noStrike">
+          <a:endParaRPr lang="en-US" sz="1100" b="0" strike="noStrike" spc="-1">
             <a:latin typeface="Times New Roman"/>
           </a:endParaRPr>
         </a:p>
@@ -1579,7 +1680,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>5</xdr:col>
@@ -1589,17 +1690,23 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>1390680</xdr:colOff>
+      <xdr:colOff>1085880</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>955080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="18" name="Image 1" descr=""/>
+        <xdr:cNvPr id="18" name="Image 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000012000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -1626,17 +1733,23 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>1381320</xdr:colOff>
+      <xdr:colOff>1089220</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>948960</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="19" name="Image 2" descr=""/>
+        <xdr:cNvPr id="19" name="Image 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000013000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -1669,11 +1782,17 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="20" name="Image 3" descr=""/>
+        <xdr:cNvPr id="20" name="Image 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000014000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId3"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -1699,18 +1818,24 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>1385640</xdr:colOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>1729</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>951840</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="21" name="Image 4" descr=""/>
+        <xdr:cNvPr id="21" name="Image 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000015000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId4"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -1737,17 +1862,23 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>1392480</xdr:colOff>
+      <xdr:colOff>1087680</xdr:colOff>
       <xdr:row>9</xdr:row>
       <xdr:rowOff>956520</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="22" name="Image 5" descr=""/>
+        <xdr:cNvPr id="22" name="Image 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000016000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId5"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -1769,54 +1900,54 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0e2841"/>
+        <a:srgbClr val="0E2841"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="e8e8e8"/>
+        <a:srgbClr val="E8E8E8"/>
       </a:lt2>
       <a:accent1>
         <a:srgbClr val="156082"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="e97132"/>
+        <a:srgbClr val="E97132"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196b24"/>
+        <a:srgbClr val="196B24"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0f9ed5"/>
+        <a:srgbClr val="0F9ED5"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="a02b93"/>
+        <a:srgbClr val="A02B93"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4ea72e"/>
+        <a:srgbClr val="4EA72E"/>
       </a:accent6>
       <a:hlink>
         <a:srgbClr val="467886"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607d"/>
+        <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -1848,7 +1979,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -1872,7 +2003,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -1932,981 +2063,964 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:L28"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="19.16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="11" min="10" style="0" width="8.37"/>
+    <col min="6" max="6" width="10.83203125" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" customWidth="1"/>
+    <col min="8" max="8" width="19.1640625" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="10" max="11" width="8.33203125" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="B2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-    </row>
-    <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-    </row>
-    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-    </row>
-    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-    </row>
-    <row r="7" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="3" t="s">
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+    </row>
+    <row r="7" spans="1:12" ht="19" x14ac:dyDescent="0.25">
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-    </row>
-    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-    </row>
-    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-    </row>
-    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-    </row>
-    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-    </row>
-    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1" t="s">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A14" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-    </row>
-    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
         <v>4</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" t="s">
         <v>5</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="C16" t="s">
         <v>6</v>
       </c>
-      <c r="D16" s="0" t="s">
+      <c r="D16" t="s">
         <v>7</v>
       </c>
-      <c r="E16" s="0" t="s">
+      <c r="E16" t="s">
         <v>8</v>
       </c>
-      <c r="F16" s="0" t="s">
+      <c r="F16" t="s">
         <v>9</v>
       </c>
-      <c r="G16" s="0" t="s">
+      <c r="G16" t="s">
         <v>10</v>
       </c>
-      <c r="H16" s="0" t="s">
+      <c r="H16" t="s">
         <v>11</v>
       </c>
-      <c r="I16" s="0" t="s">
+      <c r="I16" t="s">
         <v>12</v>
       </c>
-      <c r="J16" s="0" t="s">
+      <c r="J16" t="s">
         <v>13</v>
       </c>
-      <c r="K16" s="0" t="s">
+      <c r="K16" t="s">
         <v>14</v>
       </c>
-      <c r="L16" s="0" t="s">
+      <c r="L16" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="n">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A17" s="5">
         <v>2048</v>
       </c>
-      <c r="B17" s="4" t="n">
+      <c r="B17" s="5">
         <v>8</v>
       </c>
-      <c r="C17" s="0" t="n">
+      <c r="C17">
         <v>347.5</v>
       </c>
-      <c r="D17" s="0" t="n">
+      <c r="D17">
         <v>822.1</v>
       </c>
-      <c r="E17" s="0" t="n">
-        <v>0.285</v>
-      </c>
-      <c r="F17" s="4" t="n">
+      <c r="E17">
+        <v>0.28499999999999998</v>
+      </c>
+      <c r="F17" s="5">
         <v>512</v>
       </c>
-      <c r="G17" s="5" t="n">
-        <f aca="false">E17*F17</f>
-        <v>145.92</v>
-      </c>
-      <c r="H17" s="5" t="n">
-        <f aca="false">C17*F17/2000</f>
+      <c r="G17">
+        <f>E17*F17</f>
+        <v>145.91999999999999</v>
+      </c>
+      <c r="H17">
+        <f>C17*F17/2000</f>
         <v>88.96</v>
       </c>
-      <c r="I17" s="5" t="n">
-        <f aca="false">D17/1000</f>
-        <v>0.8221</v>
-      </c>
-      <c r="J17" s="5" t="n">
-        <f aca="false">H17*I17</f>
-        <v>73.134016</v>
-      </c>
-      <c r="K17" s="5" t="n">
-        <f aca="false">J17*2</f>
-        <v>146.268032</v>
-      </c>
-      <c r="L17" s="5" t="n">
-        <f aca="false">D17*F17/2000</f>
-        <v>210.4576</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="0" t="n">
-        <v>564.7</v>
-      </c>
-      <c r="D18" s="0" t="n">
+      <c r="I17">
+        <f t="shared" ref="I17:I28" si="0">D17/1000</f>
+        <v>0.82210000000000005</v>
+      </c>
+      <c r="J17">
+        <f t="shared" ref="J17:J28" si="1">H17*I17</f>
+        <v>73.134016000000003</v>
+      </c>
+      <c r="K17">
+        <f t="shared" ref="K17:K28" si="2">J17*2</f>
+        <v>146.26803200000001</v>
+      </c>
+      <c r="L17">
+        <f>D17*F17/2000</f>
+        <v>210.45760000000001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18">
+        <v>564.70000000000005</v>
+      </c>
+      <c r="D18">
         <v>462.5</v>
       </c>
-      <c r="E18" s="0" t="n">
+      <c r="E18">
         <v>0.26</v>
       </c>
-      <c r="F18" s="4"/>
-      <c r="G18" s="5" t="n">
-        <f aca="false">E18*F17</f>
+      <c r="F18" s="5"/>
+      <c r="G18">
+        <f>E18*F17</f>
         <v>133.12</v>
       </c>
-      <c r="H18" s="5" t="n">
-        <f aca="false">C18*F17/2000</f>
-        <v>144.5632</v>
-      </c>
-      <c r="I18" s="5" t="n">
-        <f aca="false">D18/1000</f>
-        <v>0.4625</v>
-      </c>
-      <c r="J18" s="5" t="n">
-        <f aca="false">H18*I18</f>
-        <v>66.86048</v>
-      </c>
-      <c r="K18" s="5" t="n">
-        <f aca="false">J18*2</f>
-        <v>133.72096</v>
-      </c>
-      <c r="L18" s="5" t="n">
-        <f aca="false">D18*F17/2000</f>
+      <c r="H18">
+        <f>C18*F17/2000</f>
+        <v>144.56320000000002</v>
+      </c>
+      <c r="I18">
+        <f t="shared" si="0"/>
+        <v>0.46250000000000002</v>
+      </c>
+      <c r="J18">
+        <f t="shared" si="1"/>
+        <v>66.86048000000001</v>
+      </c>
+      <c r="K18">
+        <f t="shared" si="2"/>
+        <v>133.72096000000002</v>
+      </c>
+      <c r="L18">
+        <f>D18*F17/2000</f>
         <v>118.4</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="0" t="n">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
+      <c r="C19">
         <v>999.3</v>
       </c>
-      <c r="D19" s="0" t="n">
+      <c r="D19">
         <v>284.5</v>
       </c>
-      <c r="E19" s="0" t="n">
-        <v>0.281</v>
-      </c>
-      <c r="F19" s="4"/>
-      <c r="G19" s="5" t="n">
-        <f aca="false">E19*F17</f>
-        <v>143.872</v>
-      </c>
-      <c r="H19" s="5" t="n">
-        <f aca="false">C19*F17/2000</f>
-        <v>255.8208</v>
-      </c>
-      <c r="I19" s="5" t="n">
-        <f aca="false">D19/1000</f>
-        <v>0.2845</v>
-      </c>
-      <c r="J19" s="5" t="n">
-        <f aca="false">H19*I19</f>
-        <v>72.7810176</v>
-      </c>
-      <c r="K19" s="5" t="n">
-        <f aca="false">J19*2</f>
-        <v>145.5620352</v>
-      </c>
-      <c r="L19" s="5" t="n">
-        <f aca="false">D19*F17/2000</f>
-        <v>72.832</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="n">
+      <c r="E19">
+        <v>0.28100000000000003</v>
+      </c>
+      <c r="F19" s="5"/>
+      <c r="G19">
+        <f>E19*F17</f>
+        <v>143.87200000000001</v>
+      </c>
+      <c r="H19">
+        <f>C19*F17/2000</f>
+        <v>255.82079999999999</v>
+      </c>
+      <c r="I19">
+        <f t="shared" si="0"/>
+        <v>0.28449999999999998</v>
+      </c>
+      <c r="J19">
+        <f t="shared" si="1"/>
+        <v>72.781017599999984</v>
+      </c>
+      <c r="K19">
+        <f t="shared" si="2"/>
+        <v>145.56203519999997</v>
+      </c>
+      <c r="L19">
+        <f>D19*F17/2000</f>
+        <v>72.831999999999994</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A20" s="5">
         <v>2048</v>
       </c>
-      <c r="B20" s="4" t="n">
+      <c r="B20" s="5">
         <v>16</v>
       </c>
-      <c r="C20" s="6" t="n">
-        <v>567.3</v>
-      </c>
-      <c r="D20" s="6" t="n">
+      <c r="C20" s="9">
+        <v>567.29999999999995</v>
+      </c>
+      <c r="D20" s="9">
         <v>831.1</v>
       </c>
-      <c r="E20" s="0" t="n">
-        <v>0.468</v>
-      </c>
-      <c r="F20" s="4" t="n">
+      <c r="E20">
+        <v>0.46800000000000003</v>
+      </c>
+      <c r="F20" s="5">
         <v>256</v>
       </c>
-      <c r="G20" s="5" t="n">
-        <f aca="false">E20*F20</f>
-        <v>119.808</v>
-      </c>
-      <c r="H20" s="5" t="n">
-        <f aca="false">C20*F20/2000</f>
-        <v>72.6144</v>
-      </c>
-      <c r="I20" s="5" t="n">
-        <f aca="false">D20/1000</f>
-        <v>0.8311</v>
-      </c>
-      <c r="J20" s="5" t="n">
-        <f aca="false">H20*I20</f>
-        <v>60.34982784</v>
-      </c>
-      <c r="K20" s="5" t="n">
-        <f aca="false">J20*2</f>
-        <v>120.69965568</v>
-      </c>
-      <c r="L20" s="5" t="n">
-        <f aca="false">D20*F20/2000</f>
-        <v>106.3808</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="6" t="n">
+      <c r="G20">
+        <f>E20*F20</f>
+        <v>119.80800000000001</v>
+      </c>
+      <c r="H20">
+        <f>C20*F20/2000</f>
+        <v>72.614399999999989</v>
+      </c>
+      <c r="I20">
+        <f t="shared" si="0"/>
+        <v>0.83110000000000006</v>
+      </c>
+      <c r="J20">
+        <f t="shared" si="1"/>
+        <v>60.349827839999996</v>
+      </c>
+      <c r="K20">
+        <f t="shared" si="2"/>
+        <v>120.69965567999999</v>
+      </c>
+      <c r="L20">
+        <f>D20*F20/2000</f>
+        <v>106.38080000000001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="9">
         <v>1004.3</v>
       </c>
-      <c r="D21" s="0" t="n">
+      <c r="D21">
         <v>471.4</v>
       </c>
-      <c r="E21" s="6" t="n">
-        <v>0.467</v>
-      </c>
-      <c r="F21" s="4"/>
-      <c r="G21" s="5" t="n">
-        <f aca="false">E21*F20</f>
-        <v>119.552</v>
-      </c>
-      <c r="H21" s="5" t="n">
-        <f aca="false">C21*F20/2000</f>
+      <c r="E21" s="9">
+        <v>0.46700000000000003</v>
+      </c>
+      <c r="F21" s="5"/>
+      <c r="G21">
+        <f>E21*F20</f>
+        <v>119.55200000000001</v>
+      </c>
+      <c r="H21">
+        <f>C21*F20/2000</f>
         <v>128.5504</v>
       </c>
-      <c r="I21" s="5" t="n">
-        <f aca="false">D21/1000</f>
-        <v>0.4714</v>
-      </c>
-      <c r="J21" s="5" t="n">
-        <f aca="false">H21*I21</f>
-        <v>60.59865856</v>
-      </c>
-      <c r="K21" s="5" t="n">
-        <f aca="false">J21*2</f>
-        <v>121.19731712</v>
-      </c>
-      <c r="L21" s="5" t="n">
-        <f aca="false">D21*F20/2000</f>
-        <v>60.3392</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="6" t="n">
+      <c r="I21">
+        <f t="shared" si="0"/>
+        <v>0.47139999999999999</v>
+      </c>
+      <c r="J21">
+        <f t="shared" si="1"/>
+        <v>60.598658559999997</v>
+      </c>
+      <c r="K21">
+        <f t="shared" si="2"/>
+        <v>121.19731711999999</v>
+      </c>
+      <c r="L21">
+        <f>D21*F20/2000</f>
+        <v>60.339199999999998</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="9">
         <v>1878.7</v>
       </c>
-      <c r="D22" s="6" t="n">
+      <c r="D22" s="9">
         <v>293.5</v>
       </c>
-      <c r="E22" s="6" t="n">
-        <v>0.538</v>
-      </c>
-      <c r="F22" s="4"/>
-      <c r="G22" s="5" t="n">
-        <f aca="false">E22*F20</f>
-        <v>137.728</v>
-      </c>
-      <c r="H22" s="5" t="n">
-        <f aca="false">C22*F20/2000</f>
+      <c r="E22" s="9">
+        <v>0.53800000000000003</v>
+      </c>
+      <c r="F22" s="5"/>
+      <c r="G22">
+        <f>E22*F20</f>
+        <v>137.72800000000001</v>
+      </c>
+      <c r="H22">
+        <f>C22*F20/2000</f>
         <v>240.4736</v>
       </c>
-      <c r="I22" s="5" t="n">
-        <f aca="false">D22/1000</f>
-        <v>0.2935</v>
-      </c>
-      <c r="J22" s="5" t="n">
-        <f aca="false">H22*I22</f>
-        <v>70.5790016</v>
-      </c>
-      <c r="K22" s="5" t="n">
-        <f aca="false">J22*2</f>
+      <c r="I22">
+        <f t="shared" si="0"/>
+        <v>0.29349999999999998</v>
+      </c>
+      <c r="J22">
+        <f t="shared" si="1"/>
+        <v>70.579001599999998</v>
+      </c>
+      <c r="K22">
+        <f t="shared" si="2"/>
         <v>141.1580032</v>
       </c>
-      <c r="L22" s="5" t="n">
-        <f aca="false">D22*F20/2000</f>
-        <v>37.568</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="n">
+      <c r="L22">
+        <f>D22*F20/2000</f>
+        <v>37.567999999999998</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A23" s="5">
         <v>2048</v>
       </c>
-      <c r="B23" s="4" t="n">
+      <c r="B23" s="5">
         <v>32</v>
       </c>
-      <c r="C23" s="6" t="n">
+      <c r="C23" s="9">
         <v>1007</v>
       </c>
-      <c r="D23" s="6" t="n">
+      <c r="D23" s="9">
         <v>849</v>
       </c>
-      <c r="E23" s="6" t="n">
+      <c r="E23" s="9">
         <v>0.84</v>
       </c>
-      <c r="F23" s="7" t="n">
+      <c r="F23" s="4">
         <v>128</v>
       </c>
-      <c r="G23" s="5" t="n">
-        <f aca="false">E23*F23</f>
+      <c r="G23">
+        <f>E23*F23</f>
         <v>107.52</v>
       </c>
-      <c r="H23" s="5" t="n">
-        <f aca="false">C23*F23/2000</f>
-        <v>64.448</v>
-      </c>
-      <c r="I23" s="5" t="n">
-        <f aca="false">D23/1000</f>
-        <v>0.849</v>
-      </c>
-      <c r="J23" s="5" t="n">
-        <f aca="false">H23*I23</f>
-        <v>54.716352</v>
-      </c>
-      <c r="K23" s="5" t="n">
-        <f aca="false">J23*2</f>
-        <v>109.432704</v>
-      </c>
-      <c r="L23" s="5" t="n">
-        <f aca="false">D23*F23/2000</f>
-        <v>54.336</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="6" t="n">
+      <c r="H23">
+        <f>C23*F23/2000</f>
+        <v>64.447999999999993</v>
+      </c>
+      <c r="I23">
+        <f t="shared" si="0"/>
+        <v>0.84899999999999998</v>
+      </c>
+      <c r="J23">
+        <f t="shared" si="1"/>
+        <v>54.716351999999993</v>
+      </c>
+      <c r="K23">
+        <f t="shared" si="2"/>
+        <v>109.43270399999999</v>
+      </c>
+      <c r="L23">
+        <f>D23*F23/2000</f>
+        <v>54.335999999999999</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A24" s="5"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="9">
         <v>1883.7</v>
       </c>
-      <c r="D24" s="6" t="n">
+      <c r="D24" s="9">
         <v>489.4</v>
       </c>
-      <c r="E24" s="6" t="n">
-        <v>0.892</v>
-      </c>
-      <c r="F24" s="7"/>
-      <c r="G24" s="5" t="n">
-        <f aca="false">E24*F23</f>
+      <c r="E24" s="9">
+        <v>0.89200000000000002</v>
+      </c>
+      <c r="F24" s="4"/>
+      <c r="G24">
+        <f>E24*F23</f>
         <v>114.176</v>
       </c>
-      <c r="H24" s="5" t="n">
-        <f aca="false">C24*F23/2000</f>
-        <v>120.5568</v>
-      </c>
-      <c r="I24" s="5" t="n">
-        <f aca="false">D24/1000</f>
+      <c r="H24">
+        <f>C24*F23/2000</f>
+        <v>120.55680000000001</v>
+      </c>
+      <c r="I24">
+        <f t="shared" si="0"/>
         <v>0.4894</v>
       </c>
-      <c r="J24" s="5" t="n">
-        <f aca="false">H24*I24</f>
-        <v>59.00049792</v>
-      </c>
-      <c r="K24" s="5" t="n">
-        <f aca="false">J24*2</f>
-        <v>118.00099584</v>
-      </c>
-      <c r="L24" s="5" t="n">
-        <f aca="false">D24*F23/2000</f>
+      <c r="J24">
+        <f t="shared" si="1"/>
+        <v>59.000497920000008</v>
+      </c>
+      <c r="K24">
+        <f t="shared" si="2"/>
+        <v>118.00099584000002</v>
+      </c>
+      <c r="L24">
+        <f>D24*F23/2000</f>
         <v>31.3216</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="6" t="n">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A25" s="5"/>
+      <c r="B25" s="5"/>
+      <c r="C25" s="9">
         <v>3637.4</v>
       </c>
-      <c r="D25" s="6" t="n">
-        <v>311.4</v>
-      </c>
-      <c r="E25" s="6" t="n">
-        <v>1.074</v>
-      </c>
-      <c r="F25" s="7"/>
-      <c r="G25" s="5" t="n">
-        <f aca="false">E25*F23</f>
-        <v>137.472</v>
-      </c>
-      <c r="H25" s="5" t="n">
-        <f aca="false">C25*F23/2000</f>
+      <c r="D25" s="9">
+        <v>311.39999999999998</v>
+      </c>
+      <c r="E25" s="9">
+        <v>1.0740000000000001</v>
+      </c>
+      <c r="F25" s="4"/>
+      <c r="G25">
+        <f>E25*F23</f>
+        <v>137.47200000000001</v>
+      </c>
+      <c r="H25">
+        <f>C25*F23/2000</f>
         <v>232.7936</v>
       </c>
-      <c r="I25" s="5" t="n">
-        <f aca="false">D25/1000</f>
-        <v>0.3114</v>
-      </c>
-      <c r="J25" s="5" t="n">
-        <f aca="false">H25*I25</f>
-        <v>72.49192704</v>
-      </c>
-      <c r="K25" s="5" t="n">
-        <f aca="false">J25*2</f>
-        <v>144.98385408</v>
-      </c>
-      <c r="L25" s="5" t="n">
-        <f aca="false">D25*F23/2000</f>
-        <v>19.9296</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="n">
+      <c r="I25">
+        <f t="shared" si="0"/>
+        <v>0.31139999999999995</v>
+      </c>
+      <c r="J25">
+        <f t="shared" si="1"/>
+        <v>72.491927039999993</v>
+      </c>
+      <c r="K25">
+        <f t="shared" si="2"/>
+        <v>144.98385407999999</v>
+      </c>
+      <c r="L25">
+        <f>D25*F23/2000</f>
+        <v>19.929599999999997</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A26" s="5">
         <v>2048</v>
       </c>
-      <c r="B26" s="4" t="n">
+      <c r="B26" s="5">
         <v>64</v>
       </c>
-      <c r="C26" s="6" t="n">
+      <c r="C26" s="9">
         <v>1886.4</v>
       </c>
-      <c r="D26" s="6" t="n">
+      <c r="D26" s="9">
         <v>884.9</v>
       </c>
-      <c r="E26" s="6" t="n">
-        <v>1.608</v>
-      </c>
-      <c r="F26" s="7" t="n">
+      <c r="E26" s="9">
+        <v>1.6080000000000001</v>
+      </c>
+      <c r="F26" s="4">
         <v>64</v>
       </c>
-      <c r="G26" s="5" t="n">
-        <f aca="false">E26*F26</f>
-        <v>102.912</v>
-      </c>
-      <c r="H26" s="5" t="n">
-        <f aca="false">C26*F26/2000</f>
-        <v>60.3648</v>
-      </c>
-      <c r="I26" s="5" t="n">
-        <f aca="false">D26/1000</f>
-        <v>0.8849</v>
-      </c>
-      <c r="J26" s="5" t="n">
-        <f aca="false">H26*I26</f>
-        <v>53.41681152</v>
-      </c>
-      <c r="K26" s="5" t="n">
-        <f aca="false">J26*2</f>
-        <v>106.83362304</v>
-      </c>
-      <c r="L26" s="5" t="n">
-        <f aca="false">D26*F26/2000</f>
-        <v>28.3168</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="6" t="n">
+      <c r="G26">
+        <f>E26*F26</f>
+        <v>102.91200000000001</v>
+      </c>
+      <c r="H26">
+        <f>C26*F26/2000</f>
+        <v>60.364800000000002</v>
+      </c>
+      <c r="I26">
+        <f t="shared" si="0"/>
+        <v>0.88490000000000002</v>
+      </c>
+      <c r="J26">
+        <f t="shared" si="1"/>
+        <v>53.416811520000003</v>
+      </c>
+      <c r="K26">
+        <f t="shared" si="2"/>
+        <v>106.83362304000001</v>
+      </c>
+      <c r="L26">
+        <f>D26*F26/2000</f>
+        <v>28.316800000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A27" s="5"/>
+      <c r="B27" s="5"/>
+      <c r="C27" s="9">
         <v>3642.4</v>
       </c>
-      <c r="D27" s="6" t="n">
-        <v>525.2</v>
-      </c>
-      <c r="E27" s="6" t="n">
-        <v>1.791</v>
-      </c>
-      <c r="F27" s="7"/>
-      <c r="G27" s="5" t="n">
-        <f aca="false">E27*F26</f>
+      <c r="D27" s="9">
+        <v>525.20000000000005</v>
+      </c>
+      <c r="E27" s="9">
+        <v>1.7909999999999999</v>
+      </c>
+      <c r="F27" s="4"/>
+      <c r="G27">
+        <f>E27*F26</f>
         <v>114.624</v>
       </c>
-      <c r="H27" s="5" t="n">
-        <f aca="false">C27*F26/2000</f>
-        <v>116.5568</v>
-      </c>
-      <c r="I27" s="5" t="n">
-        <f aca="false">D27/1000</f>
+      <c r="H27">
+        <f>C27*F26/2000</f>
+        <v>116.55680000000001</v>
+      </c>
+      <c r="I27">
+        <f t="shared" si="0"/>
         <v>0.5252</v>
       </c>
-      <c r="J27" s="5" t="n">
-        <f aca="false">H27*I27</f>
-        <v>61.21563136</v>
-      </c>
-      <c r="K27" s="5" t="n">
-        <f aca="false">J27*2</f>
-        <v>122.43126272</v>
-      </c>
-      <c r="L27" s="5" t="n">
-        <f aca="false">D27*F26/2000</f>
+      <c r="J27">
+        <f t="shared" si="1"/>
+        <v>61.215631360000003</v>
+      </c>
+      <c r="K27">
+        <f t="shared" si="2"/>
+        <v>122.43126272000001</v>
+      </c>
+      <c r="L27">
+        <f>D27*F26/2000</f>
         <v>16.8064</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="n">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A28" s="7">
         <v>2048</v>
       </c>
-      <c r="B28" s="2" t="n">
+      <c r="B28" s="7">
         <v>128</v>
       </c>
-      <c r="C28" s="6" t="n">
+      <c r="C28" s="9">
         <v>3645.1</v>
       </c>
-      <c r="D28" s="6" t="n">
+      <c r="D28" s="9">
         <v>956.5</v>
       </c>
-      <c r="E28" s="6" t="n">
+      <c r="E28" s="9">
         <v>3.238</v>
       </c>
-      <c r="F28" s="2" t="n">
+      <c r="F28" s="7">
         <v>32</v>
       </c>
-      <c r="G28" s="5" t="n">
-        <f aca="false">E28*F28</f>
+      <c r="G28">
+        <f>E28*F28</f>
         <v>103.616</v>
       </c>
-      <c r="H28" s="5" t="n">
-        <f aca="false">C28*F28/2000</f>
-        <v>58.3216</v>
-      </c>
-      <c r="I28" s="5" t="n">
-        <f aca="false">D28/1000</f>
-        <v>0.9565</v>
-      </c>
-      <c r="J28" s="5" t="n">
-        <f aca="false">H28*I28</f>
-        <v>55.7846104</v>
-      </c>
-      <c r="K28" s="5" t="n">
-        <f aca="false">J28*2</f>
+      <c r="H28">
+        <f>C28*F28/2000</f>
+        <v>58.321599999999997</v>
+      </c>
+      <c r="I28">
+        <f t="shared" si="0"/>
+        <v>0.95650000000000002</v>
+      </c>
+      <c r="J28">
+        <f t="shared" si="1"/>
+        <v>55.784610399999998</v>
+      </c>
+      <c r="K28">
+        <f t="shared" si="2"/>
         <v>111.5692208</v>
       </c>
-      <c r="L28" s="5" t="n">
-        <f aca="false">D28*F28/2000</f>
+      <c r="L28">
+        <f>D28*F28/2000</f>
         <v>15.304</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="A17:A19"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="F17:F19"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="F26:F27"/>
     <mergeCell ref="A20:A22"/>
     <mergeCell ref="B20:B22"/>
     <mergeCell ref="F20:F22"/>
     <mergeCell ref="A23:A25"/>
     <mergeCell ref="B23:B25"/>
     <mergeCell ref="F23:F25"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="F26:F27"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="F17:F19"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A2:E19"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="8" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-    </row>
-    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="9" t="s">
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="10" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="n">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="2">
         <v>2048</v>
       </c>
-      <c r="B5" s="10" t="n">
+      <c r="B5" s="2">
         <v>8</v>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C5" s="10">
         <v>347.5</v>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D5" s="10">
         <v>822.1</v>
       </c>
-      <c r="E5" s="9" t="n">
-        <v>0.285</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10"/>
-      <c r="B6" s="10"/>
-      <c r="C6" s="9" t="n">
-        <v>564.7</v>
-      </c>
-      <c r="D6" s="9" t="n">
+      <c r="E5" s="10">
+        <v>0.28499999999999998</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="10">
+        <v>564.70000000000005</v>
+      </c>
+      <c r="D6" s="10">
         <v>462.5</v>
       </c>
-      <c r="E6" s="9" t="n">
+      <c r="E6" s="10">
         <v>0.26</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10"/>
-      <c r="B7" s="10"/>
-      <c r="C7" s="9" t="n">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="10">
         <v>999.3</v>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="10">
         <v>284.5</v>
       </c>
-      <c r="E7" s="9" t="n">
-        <v>0.281</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="n">
+      <c r="E7" s="10">
+        <v>0.28100000000000003</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="2">
         <v>2048</v>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="2">
         <v>7</v>
       </c>
-      <c r="C8" s="9" t="n">
+      <c r="C8" s="10">
         <v>320</v>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="D8" s="10">
         <v>821</v>
       </c>
-      <c r="E8" s="9" t="n">
-        <v>0.262</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="9" t="n">
+      <c r="E8" s="10">
+        <v>0.26200000000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="10">
         <v>509.7</v>
       </c>
-      <c r="D9" s="9" t="n">
+      <c r="D9" s="10">
         <v>461.4</v>
       </c>
-      <c r="E9" s="9" t="n">
-        <v>0.234</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="9" t="n">
+      <c r="E9" s="10">
+        <v>0.23400000000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="10">
         <v>889.4</v>
       </c>
-      <c r="D10" s="9" t="n">
-        <v>283.4</v>
-      </c>
-      <c r="E10" s="9" t="n">
+      <c r="D10" s="10">
+        <v>283.39999999999998</v>
+      </c>
+      <c r="E10" s="10">
         <v>0.25</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="n">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="2">
         <v>2048</v>
       </c>
-      <c r="B11" s="10" t="n">
+      <c r="B11" s="2">
         <v>6</v>
       </c>
-      <c r="C11" s="9" t="n">
+      <c r="C11" s="10">
         <v>292.5</v>
       </c>
-      <c r="D11" s="9" t="n">
+      <c r="D11" s="10">
         <v>819.9</v>
       </c>
-      <c r="E11" s="9" t="n">
-        <v>0.239</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="n">
+      <c r="E11" s="10">
+        <v>0.23899999999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" s="2">
         <v>2048</v>
       </c>
-      <c r="B12" s="10"/>
-      <c r="C12" s="9" t="n">
+      <c r="B12" s="2"/>
+      <c r="C12" s="10">
         <v>454.7</v>
       </c>
-      <c r="D12" s="9" t="n">
+      <c r="D12" s="10">
         <v>460.2</v>
       </c>
-      <c r="E12" s="9" t="n">
-        <v>0.209</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="9" t="n">
+      <c r="E12" s="10">
+        <v>0.20899999999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="10">
         <v>779.5</v>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="D13" s="10">
         <v>282.3</v>
       </c>
-      <c r="E13" s="9" t="n">
+      <c r="E13" s="10">
         <v>0.218</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="n">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="2">
         <v>1024</v>
       </c>
-      <c r="B14" s="10" t="n">
+      <c r="B14" s="2">
         <v>16</v>
       </c>
-      <c r="C14" s="9" t="n">
-        <v>564.7</v>
-      </c>
-      <c r="D14" s="9" t="n">
+      <c r="C14" s="10">
+        <v>564.70000000000005</v>
+      </c>
+      <c r="D14" s="10">
         <v>481.7</v>
       </c>
-      <c r="E14" s="9" t="n">
-        <v>0.269</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="9" t="n">
+      <c r="E14" s="10">
+        <v>0.26900000000000002</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="10">
         <v>999.3</v>
       </c>
-      <c r="D15" s="9" t="n">
+      <c r="D15" s="10">
         <v>296.7</v>
       </c>
-      <c r="E15" s="9" t="n">
-        <v>0.29</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="9" t="n">
+      <c r="E15" s="10">
+        <v>0.28999999999999998</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="10">
         <v>1876</v>
       </c>
-      <c r="D16" s="9" t="n">
+      <c r="D16" s="10">
         <v>206.1</v>
       </c>
-      <c r="E16" s="9" t="n">
+      <c r="E16" s="10">
         <v>0.373</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="n">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="11">
         <v>2032</v>
       </c>
-      <c r="B17" s="10" t="n">
+      <c r="B17" s="11">
         <v>8</v>
       </c>
-      <c r="C17" s="9" t="n">
+      <c r="C17" s="10">
         <v>347.5</v>
       </c>
-      <c r="D17" s="9" t="n">
+      <c r="D17" s="10">
         <v>816.7</v>
       </c>
-      <c r="E17" s="9" t="n">
-        <v>0.283</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="n">
+      <c r="E17" s="10">
+        <v>0.28299999999999997</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="2">
         <v>2016</v>
       </c>
-      <c r="B18" s="10" t="n">
+      <c r="B18" s="2">
         <v>8</v>
       </c>
-      <c r="C18" s="9" t="n">
+      <c r="C18" s="10">
         <v>347.5</v>
       </c>
-      <c r="D18" s="9" t="n">
+      <c r="D18" s="10">
         <v>811.2</v>
       </c>
-      <c r="E18" s="9" t="n">
-        <v>0.281</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10"/>
-      <c r="B19" s="10"/>
-      <c r="C19" s="9" t="n">
-        <v>564.7</v>
-      </c>
-      <c r="D19" s="9" t="n">
+      <c r="E18" s="10">
+        <v>0.28100000000000003</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="10">
+        <v>564.70000000000005</v>
+      </c>
+      <c r="D19" s="10">
         <v>457</v>
       </c>
-      <c r="E19" s="9" t="n">
-        <v>0.257</v>
+      <c r="E19" s="10">
+        <v>0.25700000000000001</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="A5:A7"/>
-    <mergeCell ref="B5:B7"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="B8:B10"/>
     <mergeCell ref="A11:A13"/>
     <mergeCell ref="B11:B13"/>
     <mergeCell ref="A14:A16"/>
     <mergeCell ref="B14:B16"/>
     <mergeCell ref="A18:A19"/>
     <mergeCell ref="B18:B19"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="B8:B10"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A5:F14"/>
-  <sheetFormatPr defaultColWidth="10.4921875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A5:G14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14.39"/>
+    <col min="1" max="1" width="21.5" customWidth="1"/>
+    <col min="2" max="2" width="20.5" customWidth="1"/>
+    <col min="3" max="3" width="21" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="11" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-    </row>
-    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
         <v>18</v>
       </c>
@@ -2926,119 +3040,132 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="76.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:7" ht="76" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="10" t="s">
         <v>25</v>
       </c>
       <c r="C9" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="10" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="76.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="G9" s="15" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="76.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="10" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="D11" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="10" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="79.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+    <row r="12" spans="1:7" ht="79" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" t="s">
         <v>39</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="D12" t="s">
         <v>40</v>
       </c>
-      <c r="E12" s="14" t="n">
+      <c r="E12" s="14">
         <v>799.95</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="77.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="G12" s="15" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="77.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" t="s">
         <v>42</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" t="s">
         <v>26</v>
       </c>
-      <c r="D13" s="0" t="s">
+      <c r="D13" t="s">
         <v>43</v>
       </c>
-      <c r="E13" s="14" t="n">
+      <c r="E13" s="14">
         <v>3195.95</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="77" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="G13" s="15" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="77" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>44</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" t="s">
         <v>45</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" t="s">
         <v>46</v>
       </c>
-      <c r="D14" s="0" t="s">
+      <c r="D14" t="s">
         <v>47</v>
       </c>
-      <c r="E14" s="14" t="n">
+      <c r="E14" s="14">
         <v>729.95</v>
+      </c>
+      <c r="G14" s="15" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B5:E5"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <hyperlinks>
+    <hyperlink ref="G13" r:id="rId1" xr:uid="{51A9DE6E-7D9C-DE46-9140-682545E45ECF}"/>
+    <hyperlink ref="G12" r:id="rId2" xr:uid="{CBABC400-7277-CE49-A5B4-BC9525AFFA3E}"/>
+    <hyperlink ref="G14" r:id="rId3" xr:uid="{A022BFC9-342F-4B41-9BE4-85FB678B4D62}"/>
+    <hyperlink ref="G9" r:id="rId4" xr:uid="{50591B6B-5768-4D44-A1FC-EC71D7E504F6}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>